<commit_message>
feat: complete September 2026 sales, expenses, and B4 onboarding
- Audited and committed 30 days of B1, 26 days of B2, 30 days of B3, and 10 days of B4 sales
- Appended categorized September expenses across all 4 branches
- Created SomSaiJai_Dashboard_B4_2026.xlsx and integrated B4 across business_rules, update_dashboard, index.html, and standalone dashboard
- Quarantined capital accounts (Yamaha motorcycle ฿25k, B4 setup ฿9k) and excluded non-operating transfers
- 100% tests passing in test_render_finance, test_financial_integrity, test_expense_rules
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -133,14 +133,74 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri Light"/>
-        <a:ea typeface="Calibri Light"/>
-        <a:cs typeface="Calibri Light"/>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -192,7 +252,7 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="95000"/>
@@ -201,13 +261,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -241,6 +301,17 @@
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -295,6 +366,47 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults>
+    <a:spDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="3">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="lt1"/>
+        </a:fontRef>
+      </a:style>
+    </a:spDef>
+    <a:lnDef>
+      <a:spPr/>
+      <a:bodyPr/>
+      <a:lstStyle/>
+      <a:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </a:style>
+    </a:lnDef>
+  </a:objectDefaults>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
@@ -644,11 +756,11 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AF33"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>Som Sai Jai Cold Press Bar - September 2026</v>
+        <v>Som Sai Jai Cold Press Bar (B1) - September 2026</v>
       </c>
     </row>
     <row r="3">
@@ -677,40 +789,3021 @@
         <v>Orange</v>
       </c>
       <c r="I3" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J3" t="str">
         <v>Watermelon</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Mango</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Coconut</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Apple</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>Young Coco</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="O3" t="str">
+      <c r="R3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="P3" t="str">
+      <c r="S3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="R3" t="str">
+      <c r="U3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
+      <c r="V3" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>Used Young Coco</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Bottle Revenue (฿)</v>
+      </c>
+      <c r="AF3" t="str">
+        <v>Source Note</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C4">
+        <v>4648</v>
+      </c>
+      <c r="D4">
+        <v>2838</v>
+      </c>
+      <c r="E4">
+        <v>60</v>
+      </c>
+      <c r="F4">
+        <v>2778</v>
+      </c>
+      <c r="G4">
+        <v>1810</v>
+      </c>
+      <c r="H4">
+        <v>9</v>
+      </c>
+      <c r="I4">
+        <v>1</v>
+      </c>
+      <c r="J4">
+        <v>28</v>
+      </c>
+      <c r="K4">
+        <v>6</v>
+      </c>
+      <c r="L4">
+        <v>13</v>
+      </c>
+      <c r="M4">
+        <v>4</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4">
+        <v>61</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>9</v>
+      </c>
+      <c r="U4">
+        <v>28</v>
+      </c>
+      <c r="V4">
+        <v>6</v>
+      </c>
+      <c r="W4">
+        <v>0</v>
+      </c>
+      <c r="X4">
+        <v>0</v>
+      </c>
+      <c r="Y4">
+        <v>0</v>
+      </c>
+      <c r="Z4">
+        <v>13</v>
+      </c>
+      <c r="AA4">
+        <v>4</v>
+      </c>
+      <c r="AB4">
+        <v>0</v>
+      </c>
+      <c r="AC4">
+        <v>0</v>
+      </c>
+      <c r="AD4">
+        <v>0</v>
+      </c>
+      <c r="AE4">
+        <v>0</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_30.jpg</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>02/09/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C5">
+        <v>6764</v>
+      </c>
+      <c r="D5">
+        <v>4962</v>
+      </c>
+      <c r="E5">
+        <v>120</v>
+      </c>
+      <c r="F5">
+        <v>4842</v>
+      </c>
+      <c r="G5">
+        <v>1802</v>
+      </c>
+      <c r="H5">
+        <v>12</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>40</v>
+      </c>
+      <c r="K5">
+        <v>7</v>
+      </c>
+      <c r="L5">
+        <v>13</v>
+      </c>
+      <c r="M5">
+        <v>11</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>10</v>
+      </c>
+      <c r="P5">
+        <v>0</v>
+      </c>
+      <c r="Q5">
+        <v>93</v>
+      </c>
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>12</v>
+      </c>
+      <c r="U5">
+        <v>40</v>
+      </c>
+      <c r="V5">
+        <v>7</v>
+      </c>
+      <c r="W5">
+        <v>0</v>
+      </c>
+      <c r="X5">
+        <v>0</v>
+      </c>
+      <c r="Y5">
+        <v>0</v>
+      </c>
+      <c r="Z5">
+        <v>13</v>
+      </c>
+      <c r="AA5">
+        <v>11</v>
+      </c>
+      <c r="AB5">
+        <v>10</v>
+      </c>
+      <c r="AC5">
+        <v>0</v>
+      </c>
+      <c r="AD5">
+        <v>0</v>
+      </c>
+      <c r="AE5">
+        <v>0</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_29.jpg</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/09/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C6">
+        <v>4082</v>
+      </c>
+      <c r="D6">
+        <v>1868</v>
+      </c>
+      <c r="E6">
+        <v>60</v>
+      </c>
+      <c r="F6">
+        <v>1808</v>
+      </c>
+      <c r="G6">
+        <v>2214</v>
+      </c>
+      <c r="H6">
+        <v>12</v>
+      </c>
+      <c r="I6">
+        <v>1</v>
+      </c>
+      <c r="J6">
+        <v>20</v>
+      </c>
+      <c r="K6">
+        <v>6</v>
+      </c>
+      <c r="L6">
+        <v>9</v>
+      </c>
+      <c r="M6">
+        <v>4</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+      <c r="O6">
+        <v>0</v>
+      </c>
+      <c r="P6">
+        <v>0</v>
+      </c>
+      <c r="Q6">
+        <v>52</v>
+      </c>
+      <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
+        <v>12</v>
+      </c>
+      <c r="U6">
+        <v>20</v>
+      </c>
+      <c r="V6">
+        <v>6</v>
+      </c>
+      <c r="W6">
+        <v>0</v>
+      </c>
+      <c r="X6">
+        <v>0</v>
+      </c>
+      <c r="Y6">
+        <v>0</v>
+      </c>
+      <c r="Z6">
+        <v>9</v>
+      </c>
+      <c r="AA6">
+        <v>4</v>
+      </c>
+      <c r="AB6">
+        <v>0</v>
+      </c>
+      <c r="AC6">
+        <v>0</v>
+      </c>
+      <c r="AD6">
+        <v>0</v>
+      </c>
+      <c r="AE6">
+        <v>0</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_28.jpg</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>04/09/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C7">
+        <v>8834</v>
+      </c>
+      <c r="D7">
+        <v>5325</v>
+      </c>
+      <c r="E7">
+        <v>220</v>
+      </c>
+      <c r="F7">
+        <v>5105</v>
+      </c>
+      <c r="G7">
+        <v>3509</v>
+      </c>
+      <c r="H7">
+        <v>21</v>
+      </c>
+      <c r="I7">
+        <v>2</v>
+      </c>
+      <c r="J7">
+        <v>44</v>
+      </c>
+      <c r="K7">
+        <v>9</v>
+      </c>
+      <c r="L7">
+        <v>30</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+      <c r="O7">
+        <v>6</v>
+      </c>
+      <c r="P7">
+        <v>0</v>
+      </c>
+      <c r="Q7">
+        <v>122</v>
+      </c>
+      <c r="R7">
+        <v>0</v>
+      </c>
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>21</v>
+      </c>
+      <c r="U7">
+        <v>44</v>
+      </c>
+      <c r="V7">
+        <v>9</v>
+      </c>
+      <c r="W7">
+        <v>0</v>
+      </c>
+      <c r="X7">
+        <v>0</v>
+      </c>
+      <c r="Y7">
+        <v>0</v>
+      </c>
+      <c r="Z7">
+        <v>30</v>
+      </c>
+      <c r="AA7">
+        <v>10</v>
+      </c>
+      <c r="AB7">
+        <v>6</v>
+      </c>
+      <c r="AC7">
+        <v>0</v>
+      </c>
+      <c r="AD7">
+        <v>0</v>
+      </c>
+      <c r="AE7">
+        <v>0</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_27.jpg</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>05/09/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C8">
+        <v>6197</v>
+      </c>
+      <c r="D8">
+        <v>3474</v>
+      </c>
+      <c r="E8">
+        <v>120</v>
+      </c>
+      <c r="F8">
+        <v>3354</v>
+      </c>
+      <c r="G8">
+        <v>2723</v>
+      </c>
+      <c r="H8">
+        <v>17</v>
+      </c>
+      <c r="I8">
+        <v>1</v>
+      </c>
+      <c r="J8">
+        <v>38</v>
+      </c>
+      <c r="K8">
+        <v>5</v>
+      </c>
+      <c r="L8">
+        <v>8</v>
+      </c>
+      <c r="M8">
+        <v>10</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+      <c r="O8">
+        <v>6</v>
+      </c>
+      <c r="P8">
+        <v>0</v>
+      </c>
+      <c r="Q8">
+        <v>85</v>
+      </c>
+      <c r="R8">
+        <v>0</v>
+      </c>
+      <c r="S8">
+        <v>0</v>
+      </c>
+      <c r="T8">
+        <v>17</v>
+      </c>
+      <c r="U8">
+        <v>38</v>
+      </c>
+      <c r="V8">
+        <v>5</v>
+      </c>
+      <c r="W8">
+        <v>0</v>
+      </c>
+      <c r="X8">
+        <v>0</v>
+      </c>
+      <c r="Y8">
+        <v>0</v>
+      </c>
+      <c r="Z8">
+        <v>8</v>
+      </c>
+      <c r="AA8">
+        <v>10</v>
+      </c>
+      <c r="AB8">
+        <v>6</v>
+      </c>
+      <c r="AC8">
+        <v>0</v>
+      </c>
+      <c r="AD8">
+        <v>0</v>
+      </c>
+      <c r="AE8">
+        <v>0</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_26.jpg</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/09/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C9">
+        <v>3202</v>
+      </c>
+      <c r="D9">
+        <v>1972</v>
+      </c>
+      <c r="E9">
+        <v>60</v>
+      </c>
+      <c r="F9">
+        <v>1912</v>
+      </c>
+      <c r="G9">
+        <v>1230</v>
+      </c>
+      <c r="H9">
+        <v>8</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
+        <v>19</v>
+      </c>
+      <c r="K9">
+        <v>1</v>
+      </c>
+      <c r="L9">
+        <v>10</v>
+      </c>
+      <c r="M9">
+        <v>6</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+      <c r="O9">
+        <v>3</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>47</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
+        <v>8</v>
+      </c>
+      <c r="U9">
+        <v>19</v>
+      </c>
+      <c r="V9">
+        <v>1</v>
+      </c>
+      <c r="W9">
+        <v>0</v>
+      </c>
+      <c r="X9">
+        <v>0</v>
+      </c>
+      <c r="Y9">
+        <v>0</v>
+      </c>
+      <c r="Z9">
+        <v>10</v>
+      </c>
+      <c r="AA9">
+        <v>6</v>
+      </c>
+      <c r="AB9">
+        <v>3</v>
+      </c>
+      <c r="AC9">
+        <v>0</v>
+      </c>
+      <c r="AD9">
+        <v>0</v>
+      </c>
+      <c r="AE9">
+        <v>0</v>
+      </c>
+      <c r="AF9" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_25.jpg</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>07/09/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C10">
+        <v>5073</v>
+      </c>
+      <c r="D10">
+        <v>3239</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="F10">
+        <v>3179</v>
+      </c>
+      <c r="G10">
+        <v>1834</v>
+      </c>
+      <c r="H10">
+        <v>15</v>
+      </c>
+      <c r="I10">
+        <v>1</v>
+      </c>
+      <c r="J10">
+        <v>30</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
+      <c r="L10">
+        <v>10</v>
+      </c>
+      <c r="M10">
+        <v>7</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+      <c r="O10">
+        <v>5</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>70</v>
+      </c>
+      <c r="R10">
+        <v>0</v>
+      </c>
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
+        <v>15</v>
+      </c>
+      <c r="U10">
+        <v>30</v>
+      </c>
+      <c r="V10">
+        <v>2</v>
+      </c>
+      <c r="W10">
+        <v>0</v>
+      </c>
+      <c r="X10">
+        <v>0</v>
+      </c>
+      <c r="Y10">
+        <v>0</v>
+      </c>
+      <c r="Z10">
+        <v>10</v>
+      </c>
+      <c r="AA10">
+        <v>7</v>
+      </c>
+      <c r="AB10">
+        <v>5</v>
+      </c>
+      <c r="AC10">
+        <v>0</v>
+      </c>
+      <c r="AD10">
+        <v>0</v>
+      </c>
+      <c r="AE10">
+        <v>0</v>
+      </c>
+      <c r="AF10" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_24.jpg</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>08/09/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C11">
+        <v>5065</v>
+      </c>
+      <c r="D11">
+        <v>2303</v>
+      </c>
+      <c r="E11">
+        <v>90</v>
+      </c>
+      <c r="F11">
+        <v>2213</v>
+      </c>
+      <c r="G11">
+        <v>2762</v>
+      </c>
+      <c r="H11">
+        <v>13</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>31</v>
+      </c>
+      <c r="K11">
+        <v>3</v>
+      </c>
+      <c r="L11">
+        <v>13</v>
+      </c>
+      <c r="M11">
+        <v>2</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+      <c r="O11">
+        <v>10</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>72</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11">
+        <v>0</v>
+      </c>
+      <c r="T11">
+        <v>13</v>
+      </c>
+      <c r="U11">
+        <v>31</v>
+      </c>
+      <c r="V11">
+        <v>3</v>
+      </c>
+      <c r="W11">
+        <v>0</v>
+      </c>
+      <c r="X11">
+        <v>0</v>
+      </c>
+      <c r="Y11">
+        <v>0</v>
+      </c>
+      <c r="Z11">
+        <v>13</v>
+      </c>
+      <c r="AA11">
+        <v>2</v>
+      </c>
+      <c r="AB11">
+        <v>10</v>
+      </c>
+      <c r="AC11">
+        <v>0</v>
+      </c>
+      <c r="AD11">
+        <v>0</v>
+      </c>
+      <c r="AE11">
+        <v>0</v>
+      </c>
+      <c r="AF11" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_23.jpg</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/09/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C12">
+        <v>4878</v>
+      </c>
+      <c r="D12">
+        <v>3013</v>
+      </c>
+      <c r="E12">
+        <v>60</v>
+      </c>
+      <c r="F12">
+        <v>2953</v>
+      </c>
+      <c r="G12">
+        <v>1865</v>
+      </c>
+      <c r="H12">
+        <v>19</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>30</v>
+      </c>
+      <c r="K12">
+        <v>5</v>
+      </c>
+      <c r="L12">
+        <v>7</v>
+      </c>
+      <c r="M12">
+        <v>3</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+      <c r="O12">
+        <v>3</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>67</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>19</v>
+      </c>
+      <c r="U12">
+        <v>30</v>
+      </c>
+      <c r="V12">
+        <v>5</v>
+      </c>
+      <c r="W12">
+        <v>0</v>
+      </c>
+      <c r="X12">
+        <v>0</v>
+      </c>
+      <c r="Y12">
+        <v>0</v>
+      </c>
+      <c r="Z12">
+        <v>7</v>
+      </c>
+      <c r="AA12">
+        <v>3</v>
+      </c>
+      <c r="AB12">
+        <v>3</v>
+      </c>
+      <c r="AC12">
+        <v>0</v>
+      </c>
+      <c r="AD12">
+        <v>0</v>
+      </c>
+      <c r="AE12">
+        <v>0</v>
+      </c>
+      <c r="AF12" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_22.jpg</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>10/09/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C13">
+        <v>1989</v>
+      </c>
+      <c r="D13">
+        <v>964</v>
+      </c>
+      <c r="E13">
+        <v>60</v>
+      </c>
+      <c r="F13">
+        <v>904</v>
+      </c>
+      <c r="G13">
+        <v>1025</v>
+      </c>
+      <c r="H13">
+        <v>10</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>12</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>3</v>
+      </c>
+      <c r="M13">
+        <v>2</v>
+      </c>
+      <c r="N13">
+        <v>0</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>28</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>10</v>
+      </c>
+      <c r="U13">
+        <v>12</v>
+      </c>
+      <c r="V13">
+        <v>0</v>
+      </c>
+      <c r="W13">
+        <v>0</v>
+      </c>
+      <c r="X13">
+        <v>0</v>
+      </c>
+      <c r="Y13">
+        <v>0</v>
+      </c>
+      <c r="Z13">
+        <v>3</v>
+      </c>
+      <c r="AA13">
+        <v>2</v>
+      </c>
+      <c r="AB13">
+        <v>1</v>
+      </c>
+      <c r="AC13">
+        <v>0</v>
+      </c>
+      <c r="AD13">
+        <v>0</v>
+      </c>
+      <c r="AE13">
+        <v>0</v>
+      </c>
+      <c r="AF13" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_21.jpg</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>11/09/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C14">
+        <v>2247</v>
+      </c>
+      <c r="D14">
+        <v>1267</v>
+      </c>
+      <c r="E14">
+        <v>60</v>
+      </c>
+      <c r="F14">
+        <v>1207</v>
+      </c>
+      <c r="G14">
+        <v>980</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
+      </c>
+      <c r="I14">
+        <v>0</v>
+      </c>
+      <c r="J14">
+        <v>12</v>
+      </c>
+      <c r="K14">
+        <v>2</v>
+      </c>
+      <c r="L14">
+        <v>6</v>
+      </c>
+      <c r="M14">
+        <v>4</v>
+      </c>
+      <c r="N14">
+        <v>0</v>
+      </c>
+      <c r="O14">
+        <v>3</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>31</v>
+      </c>
+      <c r="R14">
+        <v>0</v>
+      </c>
+      <c r="S14">
+        <v>0</v>
+      </c>
+      <c r="T14">
+        <v>4</v>
+      </c>
+      <c r="U14">
+        <v>12</v>
+      </c>
+      <c r="V14">
+        <v>2</v>
+      </c>
+      <c r="W14">
+        <v>0</v>
+      </c>
+      <c r="X14">
+        <v>0</v>
+      </c>
+      <c r="Y14">
+        <v>0</v>
+      </c>
+      <c r="Z14">
+        <v>6</v>
+      </c>
+      <c r="AA14">
+        <v>4</v>
+      </c>
+      <c r="AB14">
+        <v>3</v>
+      </c>
+      <c r="AC14">
+        <v>0</v>
+      </c>
+      <c r="AD14">
+        <v>0</v>
+      </c>
+      <c r="AE14">
+        <v>0</v>
+      </c>
+      <c r="AF14" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_20.jpg</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>12/09/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C15">
+        <v>5156</v>
+      </c>
+      <c r="D15">
+        <v>2640</v>
+      </c>
+      <c r="E15">
+        <v>120</v>
+      </c>
+      <c r="F15">
+        <v>2520</v>
+      </c>
+      <c r="G15">
+        <v>2516</v>
+      </c>
+      <c r="H15">
+        <v>9</v>
+      </c>
+      <c r="I15">
+        <v>0</v>
+      </c>
+      <c r="J15">
+        <v>41</v>
+      </c>
+      <c r="K15">
+        <v>4</v>
+      </c>
+      <c r="L15">
+        <v>9</v>
+      </c>
+      <c r="M15">
+        <v>3</v>
+      </c>
+      <c r="N15">
+        <v>0</v>
+      </c>
+      <c r="O15">
+        <v>7</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>73</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>9</v>
+      </c>
+      <c r="U15">
+        <v>41</v>
+      </c>
+      <c r="V15">
+        <v>4</v>
+      </c>
+      <c r="W15">
+        <v>0</v>
+      </c>
+      <c r="X15">
+        <v>0</v>
+      </c>
+      <c r="Y15">
+        <v>0</v>
+      </c>
+      <c r="Z15">
+        <v>9</v>
+      </c>
+      <c r="AA15">
+        <v>3</v>
+      </c>
+      <c r="AB15">
+        <v>7</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>0</v>
+      </c>
+      <c r="AE15">
+        <v>0</v>
+      </c>
+      <c r="AF15" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_19.jpg</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>13/09/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C16">
+        <v>7697</v>
+      </c>
+      <c r="D16">
+        <v>3938</v>
+      </c>
+      <c r="E16">
+        <v>120</v>
+      </c>
+      <c r="F16">
+        <v>3818</v>
+      </c>
+      <c r="G16">
+        <v>3759</v>
+      </c>
+      <c r="H16">
+        <v>18</v>
+      </c>
+      <c r="I16">
+        <v>0</v>
+      </c>
+      <c r="J16">
+        <v>53</v>
+      </c>
+      <c r="K16">
+        <v>7</v>
+      </c>
+      <c r="L16">
+        <v>12</v>
+      </c>
+      <c r="M16">
+        <v>3</v>
+      </c>
+      <c r="N16">
+        <v>0</v>
+      </c>
+      <c r="O16">
+        <v>10</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>103</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>18</v>
+      </c>
+      <c r="U16">
+        <v>53</v>
+      </c>
+      <c r="V16">
+        <v>7</v>
+      </c>
+      <c r="W16">
+        <v>0</v>
+      </c>
+      <c r="X16">
+        <v>0</v>
+      </c>
+      <c r="Y16">
+        <v>0</v>
+      </c>
+      <c r="Z16">
+        <v>12</v>
+      </c>
+      <c r="AA16">
+        <v>3</v>
+      </c>
+      <c r="AB16">
+        <v>10</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>0</v>
+      </c>
+      <c r="AE16">
+        <v>0</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_18.jpg</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>14/09/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C17">
+        <v>4868</v>
+      </c>
+      <c r="D17">
+        <v>3200</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="F17">
+        <v>3140</v>
+      </c>
+      <c r="G17">
+        <v>1668</v>
+      </c>
+      <c r="H17">
+        <v>12</v>
+      </c>
+      <c r="I17">
+        <v>2</v>
+      </c>
+      <c r="J17">
+        <v>30</v>
+      </c>
+      <c r="K17">
+        <v>4</v>
+      </c>
+      <c r="L17">
+        <v>11</v>
+      </c>
+      <c r="M17">
+        <v>5</v>
+      </c>
+      <c r="N17">
+        <v>0</v>
+      </c>
+      <c r="O17">
+        <v>4</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>68</v>
+      </c>
+      <c r="R17">
+        <v>0</v>
+      </c>
+      <c r="S17">
+        <v>0</v>
+      </c>
+      <c r="T17">
+        <v>12</v>
+      </c>
+      <c r="U17">
+        <v>30</v>
+      </c>
+      <c r="V17">
+        <v>4</v>
+      </c>
+      <c r="W17">
+        <v>0</v>
+      </c>
+      <c r="X17">
+        <v>0</v>
+      </c>
+      <c r="Y17">
+        <v>0</v>
+      </c>
+      <c r="Z17">
+        <v>11</v>
+      </c>
+      <c r="AA17">
+        <v>5</v>
+      </c>
+      <c r="AB17">
+        <v>4</v>
+      </c>
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>0</v>
+      </c>
+      <c r="AE17">
+        <v>0</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_17.jpg</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>15/09/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C18">
+        <v>1154</v>
+      </c>
+      <c r="D18">
+        <v>685</v>
+      </c>
+      <c r="E18">
+        <v>60</v>
+      </c>
+      <c r="F18">
+        <v>625</v>
+      </c>
+      <c r="G18">
+        <v>469</v>
+      </c>
+      <c r="H18">
+        <v>2</v>
+      </c>
+      <c r="I18">
+        <v>0</v>
+      </c>
+      <c r="J18">
+        <v>5</v>
+      </c>
+      <c r="K18">
+        <v>2</v>
+      </c>
+      <c r="L18">
+        <v>1</v>
+      </c>
+      <c r="M18">
+        <v>3</v>
+      </c>
+      <c r="N18">
+        <v>0</v>
+      </c>
+      <c r="O18">
+        <v>3</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>16</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>2</v>
+      </c>
+      <c r="U18">
+        <v>5</v>
+      </c>
+      <c r="V18">
+        <v>2</v>
+      </c>
+      <c r="W18">
+        <v>0</v>
+      </c>
+      <c r="X18">
+        <v>0</v>
+      </c>
+      <c r="Y18">
+        <v>0</v>
+      </c>
+      <c r="Z18">
+        <v>1</v>
+      </c>
+      <c r="AA18">
+        <v>3</v>
+      </c>
+      <c r="AB18">
+        <v>3</v>
+      </c>
+      <c r="AC18">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>0</v>
+      </c>
+      <c r="AE18">
+        <v>0</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_16.jpg</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>16/09/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C19">
+        <v>1603</v>
+      </c>
+      <c r="D19">
+        <v>1198</v>
+      </c>
+      <c r="E19">
+        <v>60</v>
+      </c>
+      <c r="F19">
+        <v>1138</v>
+      </c>
+      <c r="G19">
+        <v>405</v>
+      </c>
+      <c r="H19">
+        <v>1</v>
+      </c>
+      <c r="I19">
+        <v>0</v>
+      </c>
+      <c r="J19">
+        <v>7</v>
+      </c>
+      <c r="K19">
+        <v>6</v>
+      </c>
+      <c r="L19">
+        <v>5</v>
+      </c>
+      <c r="M19">
+        <v>1</v>
+      </c>
+      <c r="N19">
+        <v>0</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>20</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
+      </c>
+      <c r="S19">
+        <v>0</v>
+      </c>
+      <c r="T19">
+        <v>1</v>
+      </c>
+      <c r="U19">
+        <v>7</v>
+      </c>
+      <c r="V19">
+        <v>6</v>
+      </c>
+      <c r="W19">
+        <v>0</v>
+      </c>
+      <c r="X19">
+        <v>0</v>
+      </c>
+      <c r="Y19">
+        <v>0</v>
+      </c>
+      <c r="Z19">
+        <v>5</v>
+      </c>
+      <c r="AA19">
+        <v>1</v>
+      </c>
+      <c r="AB19">
+        <v>0</v>
+      </c>
+      <c r="AC19">
+        <v>0</v>
+      </c>
+      <c r="AD19">
+        <v>0</v>
+      </c>
+      <c r="AE19">
+        <v>0</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_15.jpg</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>17/09/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C20">
+        <v>2144</v>
+      </c>
+      <c r="D20">
+        <v>1280</v>
+      </c>
+      <c r="E20">
+        <v>111</v>
+      </c>
+      <c r="F20">
+        <v>1169</v>
+      </c>
+      <c r="G20">
+        <v>864</v>
+      </c>
+      <c r="H20">
+        <v>10</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <v>0</v>
+      </c>
+      <c r="K20">
+        <v>0</v>
+      </c>
+      <c r="L20">
+        <v>11</v>
+      </c>
+      <c r="M20">
+        <v>5</v>
+      </c>
+      <c r="N20">
+        <v>0</v>
+      </c>
+      <c r="O20">
+        <v>2</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>29</v>
+      </c>
+      <c r="R20">
+        <v>0</v>
+      </c>
+      <c r="S20">
+        <v>0</v>
+      </c>
+      <c r="T20">
+        <v>10</v>
+      </c>
+      <c r="U20">
+        <v>0</v>
+      </c>
+      <c r="V20">
+        <v>0</v>
+      </c>
+      <c r="W20">
+        <v>0</v>
+      </c>
+      <c r="X20">
+        <v>0</v>
+      </c>
+      <c r="Y20">
+        <v>0</v>
+      </c>
+      <c r="Z20">
+        <v>11</v>
+      </c>
+      <c r="AA20">
+        <v>5</v>
+      </c>
+      <c r="AB20">
+        <v>2</v>
+      </c>
+      <c r="AC20">
+        <v>0</v>
+      </c>
+      <c r="AD20">
+        <v>0</v>
+      </c>
+      <c r="AE20">
+        <v>0</v>
+      </c>
+      <c r="AF20" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_14.jpg</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>18/09/2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C21">
+        <v>5190</v>
+      </c>
+      <c r="D21">
+        <v>2910</v>
+      </c>
+      <c r="E21">
+        <v>120</v>
+      </c>
+      <c r="F21">
+        <v>2790</v>
+      </c>
+      <c r="G21">
+        <v>2280</v>
+      </c>
+      <c r="H21">
+        <v>14</v>
+      </c>
+      <c r="I21">
+        <v>0</v>
+      </c>
+      <c r="J21">
+        <v>0</v>
+      </c>
+      <c r="K21">
+        <v>3</v>
+      </c>
+      <c r="L21">
+        <v>20</v>
+      </c>
+      <c r="M21">
+        <v>25</v>
+      </c>
+      <c r="N21">
+        <v>0</v>
+      </c>
+      <c r="O21">
+        <v>10</v>
+      </c>
+      <c r="P21">
+        <v>0</v>
+      </c>
+      <c r="Q21">
+        <v>73</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>14</v>
+      </c>
+      <c r="U21">
+        <v>0</v>
+      </c>
+      <c r="V21">
+        <v>3</v>
+      </c>
+      <c r="W21">
+        <v>0</v>
+      </c>
+      <c r="X21">
+        <v>0</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <v>20</v>
+      </c>
+      <c r="AA21">
+        <v>25</v>
+      </c>
+      <c r="AB21">
+        <v>10</v>
+      </c>
+      <c r="AC21">
+        <v>0</v>
+      </c>
+      <c r="AD21">
+        <v>0</v>
+      </c>
+      <c r="AE21">
+        <v>0</v>
+      </c>
+      <c r="AF21" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_13.jpg</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>19/09/2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C22">
+        <v>3470</v>
+      </c>
+      <c r="D22">
+        <v>2110</v>
+      </c>
+      <c r="E22">
+        <v>120</v>
+      </c>
+      <c r="F22">
+        <v>1990</v>
+      </c>
+      <c r="G22">
+        <v>1360</v>
+      </c>
+      <c r="H22">
+        <v>9</v>
+      </c>
+      <c r="I22">
+        <v>0</v>
+      </c>
+      <c r="J22">
+        <v>11</v>
+      </c>
+      <c r="K22">
+        <v>6</v>
+      </c>
+      <c r="L22">
+        <v>12</v>
+      </c>
+      <c r="M22">
+        <v>4</v>
+      </c>
+      <c r="N22">
+        <v>0</v>
+      </c>
+      <c r="O22">
+        <v>6</v>
+      </c>
+      <c r="P22">
+        <v>0</v>
+      </c>
+      <c r="Q22">
+        <v>48</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>9</v>
+      </c>
+      <c r="U22">
+        <v>11</v>
+      </c>
+      <c r="V22">
+        <v>6</v>
+      </c>
+      <c r="W22">
+        <v>0</v>
+      </c>
+      <c r="X22">
+        <v>0</v>
+      </c>
+      <c r="Y22">
+        <v>0</v>
+      </c>
+      <c r="Z22">
+        <v>12</v>
+      </c>
+      <c r="AA22">
+        <v>4</v>
+      </c>
+      <c r="AB22">
+        <v>6</v>
+      </c>
+      <c r="AC22">
+        <v>0</v>
+      </c>
+      <c r="AD22">
+        <v>0</v>
+      </c>
+      <c r="AE22">
+        <v>0</v>
+      </c>
+      <c r="AF22" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_12.jpg</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>20/09/2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C23">
+        <v>1030</v>
+      </c>
+      <c r="D23">
+        <v>680</v>
+      </c>
+      <c r="E23">
+        <v>60</v>
+      </c>
+      <c r="F23">
+        <v>620</v>
+      </c>
+      <c r="G23">
+        <v>350</v>
+      </c>
+      <c r="H23">
+        <v>2</v>
+      </c>
+      <c r="I23">
+        <v>0</v>
+      </c>
+      <c r="J23">
+        <v>0</v>
+      </c>
+      <c r="K23">
+        <v>1</v>
+      </c>
+      <c r="L23">
+        <v>8</v>
+      </c>
+      <c r="M23">
+        <v>3</v>
+      </c>
+      <c r="N23">
+        <v>0</v>
+      </c>
+      <c r="O23">
+        <v>1</v>
+      </c>
+      <c r="P23">
+        <v>0</v>
+      </c>
+      <c r="Q23">
+        <v>15</v>
+      </c>
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>2</v>
+      </c>
+      <c r="U23">
+        <v>0</v>
+      </c>
+      <c r="V23">
+        <v>1</v>
+      </c>
+      <c r="W23">
+        <v>0</v>
+      </c>
+      <c r="X23">
+        <v>0</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="Z23">
+        <v>8</v>
+      </c>
+      <c r="AA23">
+        <v>3</v>
+      </c>
+      <c r="AB23">
+        <v>1</v>
+      </c>
+      <c r="AC23">
+        <v>0</v>
+      </c>
+      <c r="AD23">
+        <v>0</v>
+      </c>
+      <c r="AE23">
+        <v>0</v>
+      </c>
+      <c r="AF23" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_11.jpg</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>21/09/2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C24">
+        <v>2617</v>
+      </c>
+      <c r="D24">
+        <v>2087</v>
+      </c>
+      <c r="E24">
+        <v>60</v>
+      </c>
+      <c r="F24">
+        <v>2027</v>
+      </c>
+      <c r="G24">
+        <v>530</v>
+      </c>
+      <c r="H24">
+        <v>0</v>
+      </c>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <v>19</v>
+      </c>
+      <c r="K24">
+        <v>0</v>
+      </c>
+      <c r="L24">
+        <v>10</v>
+      </c>
+      <c r="M24">
+        <v>8</v>
+      </c>
+      <c r="N24">
+        <v>0</v>
+      </c>
+      <c r="O24">
+        <v>4</v>
+      </c>
+      <c r="P24">
+        <v>0</v>
+      </c>
+      <c r="Q24">
+        <v>41</v>
+      </c>
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+      <c r="U24">
+        <v>19</v>
+      </c>
+      <c r="V24">
+        <v>0</v>
+      </c>
+      <c r="W24">
+        <v>0</v>
+      </c>
+      <c r="X24">
+        <v>0</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24">
+        <v>10</v>
+      </c>
+      <c r="AA24">
+        <v>8</v>
+      </c>
+      <c r="AB24">
+        <v>4</v>
+      </c>
+      <c r="AC24">
+        <v>0</v>
+      </c>
+      <c r="AD24">
+        <v>0</v>
+      </c>
+      <c r="AE24">
+        <v>0</v>
+      </c>
+      <c r="AF24" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_10.jpg</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C25">
+        <v>4748</v>
+      </c>
+      <c r="D25">
+        <v>1570</v>
+      </c>
+      <c r="E25">
+        <v>120</v>
+      </c>
+      <c r="F25">
+        <v>1450</v>
+      </c>
+      <c r="G25">
+        <v>3178</v>
+      </c>
+      <c r="H25">
+        <v>12</v>
+      </c>
+      <c r="I25">
+        <v>0</v>
+      </c>
+      <c r="J25">
+        <v>0</v>
+      </c>
+      <c r="K25">
+        <v>2</v>
+      </c>
+      <c r="L25">
+        <v>29</v>
+      </c>
+      <c r="M25">
+        <v>12</v>
+      </c>
+      <c r="N25">
+        <v>0</v>
+      </c>
+      <c r="O25">
+        <v>6</v>
+      </c>
+      <c r="P25">
+        <v>0</v>
+      </c>
+      <c r="Q25">
+        <v>61</v>
+      </c>
+      <c r="R25">
+        <v>0</v>
+      </c>
+      <c r="S25">
+        <v>0</v>
+      </c>
+      <c r="T25">
+        <v>12</v>
+      </c>
+      <c r="U25">
+        <v>0</v>
+      </c>
+      <c r="V25">
+        <v>2</v>
+      </c>
+      <c r="W25">
+        <v>0</v>
+      </c>
+      <c r="X25">
+        <v>0</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <v>29</v>
+      </c>
+      <c r="AA25">
+        <v>12</v>
+      </c>
+      <c r="AB25">
+        <v>6</v>
+      </c>
+      <c r="AC25">
+        <v>0</v>
+      </c>
+      <c r="AD25">
+        <v>0</v>
+      </c>
+      <c r="AE25">
+        <v>0</v>
+      </c>
+      <c r="AF25" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_8.jpg</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>23/09/2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C26">
+        <v>4327</v>
+      </c>
+      <c r="D26">
+        <v>2787</v>
+      </c>
+      <c r="E26">
+        <v>244</v>
+      </c>
+      <c r="F26">
+        <v>2543</v>
+      </c>
+      <c r="G26">
+        <v>1540</v>
+      </c>
+      <c r="H26">
+        <v>6</v>
+      </c>
+      <c r="I26">
+        <v>0</v>
+      </c>
+      <c r="J26">
+        <v>0</v>
+      </c>
+      <c r="K26">
+        <v>10</v>
+      </c>
+      <c r="L26">
+        <v>28</v>
+      </c>
+      <c r="M26">
+        <v>4</v>
+      </c>
+      <c r="N26">
+        <v>0</v>
+      </c>
+      <c r="O26">
+        <v>9</v>
+      </c>
+      <c r="P26">
+        <v>0</v>
+      </c>
+      <c r="Q26">
+        <v>57</v>
+      </c>
+      <c r="R26">
+        <v>0</v>
+      </c>
+      <c r="S26">
+        <v>0</v>
+      </c>
+      <c r="T26">
+        <v>6</v>
+      </c>
+      <c r="U26">
+        <v>0</v>
+      </c>
+      <c r="V26">
+        <v>10</v>
+      </c>
+      <c r="W26">
+        <v>0</v>
+      </c>
+      <c r="X26">
+        <v>0</v>
+      </c>
+      <c r="Y26">
+        <v>0</v>
+      </c>
+      <c r="Z26">
+        <v>28</v>
+      </c>
+      <c r="AA26">
+        <v>4</v>
+      </c>
+      <c r="AB26">
+        <v>9</v>
+      </c>
+      <c r="AC26">
+        <v>0</v>
+      </c>
+      <c r="AD26">
+        <v>0</v>
+      </c>
+      <c r="AE26">
+        <v>0</v>
+      </c>
+      <c r="AF26" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_9.jpg</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C27">
+        <v>3280</v>
+      </c>
+      <c r="D27">
+        <v>2225</v>
+      </c>
+      <c r="E27">
+        <v>80</v>
+      </c>
+      <c r="F27">
+        <v>2145</v>
+      </c>
+      <c r="G27">
+        <v>1055</v>
+      </c>
+      <c r="H27">
+        <v>9</v>
+      </c>
+      <c r="I27">
+        <v>0</v>
+      </c>
+      <c r="J27">
+        <v>15</v>
+      </c>
+      <c r="K27">
+        <v>2</v>
+      </c>
+      <c r="L27">
+        <v>6</v>
+      </c>
+      <c r="M27">
+        <v>9</v>
+      </c>
+      <c r="N27">
+        <v>0</v>
+      </c>
+      <c r="O27">
+        <v>5</v>
+      </c>
+      <c r="P27">
+        <v>0</v>
+      </c>
+      <c r="Q27">
+        <v>47</v>
+      </c>
+      <c r="R27">
+        <v>0</v>
+      </c>
+      <c r="S27">
+        <v>0</v>
+      </c>
+      <c r="T27">
+        <v>9</v>
+      </c>
+      <c r="U27">
+        <v>15</v>
+      </c>
+      <c r="V27">
+        <v>2</v>
+      </c>
+      <c r="W27">
+        <v>0</v>
+      </c>
+      <c r="X27">
+        <v>0</v>
+      </c>
+      <c r="Y27">
+        <v>0</v>
+      </c>
+      <c r="Z27">
+        <v>6</v>
+      </c>
+      <c r="AA27">
+        <v>9</v>
+      </c>
+      <c r="AB27">
+        <v>5</v>
+      </c>
+      <c r="AC27">
+        <v>0</v>
+      </c>
+      <c r="AD27">
+        <v>0</v>
+      </c>
+      <c r="AE27">
+        <v>0</v>
+      </c>
+      <c r="AF27" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_6.jpg</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>25/09/2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C28">
+        <v>360</v>
+      </c>
+      <c r="D28">
+        <v>360</v>
+      </c>
+      <c r="E28">
+        <v>60</v>
+      </c>
+      <c r="F28">
+        <v>300</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28">
+        <v>1</v>
+      </c>
+      <c r="I28">
+        <v>0</v>
+      </c>
+      <c r="J28">
+        <v>4</v>
+      </c>
+      <c r="K28">
+        <v>0</v>
+      </c>
+      <c r="L28">
+        <v>1</v>
+      </c>
+      <c r="M28">
+        <v>0</v>
+      </c>
+      <c r="N28">
+        <v>0</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>0</v>
+      </c>
+      <c r="Q28">
+        <v>6</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28">
+        <v>1</v>
+      </c>
+      <c r="U28">
+        <v>4</v>
+      </c>
+      <c r="V28">
+        <v>0</v>
+      </c>
+      <c r="W28">
+        <v>0</v>
+      </c>
+      <c r="X28">
+        <v>0</v>
+      </c>
+      <c r="Y28">
+        <v>0</v>
+      </c>
+      <c r="Z28">
+        <v>1</v>
+      </c>
+      <c r="AA28">
+        <v>0</v>
+      </c>
+      <c r="AB28">
+        <v>0</v>
+      </c>
+      <c r="AC28">
+        <v>0</v>
+      </c>
+      <c r="AD28">
+        <v>0</v>
+      </c>
+      <c r="AE28">
+        <v>0</v>
+      </c>
+      <c r="AF28" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_7.jpg</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>26/09/2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C29">
+        <v>7392</v>
+      </c>
+      <c r="D29">
+        <v>5392</v>
+      </c>
+      <c r="E29">
+        <v>90</v>
+      </c>
+      <c r="F29">
+        <v>5302</v>
+      </c>
+      <c r="G29">
+        <v>2000</v>
+      </c>
+      <c r="H29">
+        <v>16</v>
+      </c>
+      <c r="I29">
+        <v>0</v>
+      </c>
+      <c r="J29">
+        <v>34</v>
+      </c>
+      <c r="K29">
+        <v>9</v>
+      </c>
+      <c r="L29">
+        <v>14</v>
+      </c>
+      <c r="M29">
+        <v>15</v>
+      </c>
+      <c r="N29">
+        <v>0</v>
+      </c>
+      <c r="O29">
+        <v>11</v>
+      </c>
+      <c r="P29">
+        <v>0</v>
+      </c>
+      <c r="Q29">
+        <v>99</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>16</v>
+      </c>
+      <c r="U29">
+        <v>34</v>
+      </c>
+      <c r="V29">
+        <v>9</v>
+      </c>
+      <c r="W29">
+        <v>0</v>
+      </c>
+      <c r="X29">
+        <v>0</v>
+      </c>
+      <c r="Y29">
+        <v>0</v>
+      </c>
+      <c r="Z29">
+        <v>14</v>
+      </c>
+      <c r="AA29">
+        <v>15</v>
+      </c>
+      <c r="AB29">
+        <v>11</v>
+      </c>
+      <c r="AC29">
+        <v>0</v>
+      </c>
+      <c r="AD29">
+        <v>0</v>
+      </c>
+      <c r="AE29">
+        <v>0</v>
+      </c>
+      <c r="AF29" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_5.jpg</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>27/09/2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C30">
+        <v>5799</v>
+      </c>
+      <c r="D30">
+        <v>4620</v>
+      </c>
+      <c r="E30">
+        <v>120</v>
+      </c>
+      <c r="F30">
+        <v>4500</v>
+      </c>
+      <c r="G30">
+        <v>1179</v>
+      </c>
+      <c r="H30">
+        <v>20</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <v>23</v>
+      </c>
+      <c r="K30">
+        <v>4</v>
+      </c>
+      <c r="L30">
+        <v>9</v>
+      </c>
+      <c r="M30">
+        <v>12</v>
+      </c>
+      <c r="N30">
+        <v>0</v>
+      </c>
+      <c r="O30">
+        <v>9</v>
+      </c>
+      <c r="P30">
+        <v>0</v>
+      </c>
+      <c r="Q30">
+        <v>77</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>20</v>
+      </c>
+      <c r="U30">
+        <v>23</v>
+      </c>
+      <c r="V30">
+        <v>4</v>
+      </c>
+      <c r="W30">
+        <v>0</v>
+      </c>
+      <c r="X30">
+        <v>0</v>
+      </c>
+      <c r="Y30">
+        <v>0</v>
+      </c>
+      <c r="Z30">
+        <v>9</v>
+      </c>
+      <c r="AA30">
+        <v>12</v>
+      </c>
+      <c r="AB30">
+        <v>9</v>
+      </c>
+      <c r="AC30">
+        <v>0</v>
+      </c>
+      <c r="AD30">
+        <v>0</v>
+      </c>
+      <c r="AE30">
+        <v>0</v>
+      </c>
+      <c r="AF30" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_4.jpg</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>28/09/2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C31">
+        <v>5789</v>
+      </c>
+      <c r="D31">
+        <v>4550</v>
+      </c>
+      <c r="E31">
+        <v>60</v>
+      </c>
+      <c r="F31">
+        <v>4490</v>
+      </c>
+      <c r="G31">
+        <v>1239</v>
+      </c>
+      <c r="H31">
+        <v>12</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <v>30</v>
+      </c>
+      <c r="K31">
+        <v>4</v>
+      </c>
+      <c r="L31">
+        <v>5</v>
+      </c>
+      <c r="M31">
+        <v>8</v>
+      </c>
+      <c r="N31">
+        <v>0</v>
+      </c>
+      <c r="O31">
+        <v>12</v>
+      </c>
+      <c r="P31">
+        <v>0</v>
+      </c>
+      <c r="Q31">
+        <v>71</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>12</v>
+      </c>
+      <c r="U31">
+        <v>30</v>
+      </c>
+      <c r="V31">
+        <v>4</v>
+      </c>
+      <c r="W31">
+        <v>0</v>
+      </c>
+      <c r="X31">
+        <v>0</v>
+      </c>
+      <c r="Y31">
+        <v>0</v>
+      </c>
+      <c r="Z31">
+        <v>5</v>
+      </c>
+      <c r="AA31">
+        <v>8</v>
+      </c>
+      <c r="AB31">
+        <v>12</v>
+      </c>
+      <c r="AC31">
+        <v>0</v>
+      </c>
+      <c r="AD31">
+        <v>0</v>
+      </c>
+      <c r="AE31">
+        <v>0</v>
+      </c>
+      <c r="AF31" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_3.jpg</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>29/09/2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C32">
+        <v>5123</v>
+      </c>
+      <c r="D32">
+        <v>3234</v>
+      </c>
+      <c r="E32">
+        <v>120</v>
+      </c>
+      <c r="F32">
+        <v>3114</v>
+      </c>
+      <c r="G32">
+        <v>1889</v>
+      </c>
+      <c r="H32">
+        <v>16</v>
+      </c>
+      <c r="I32">
+        <v>0</v>
+      </c>
+      <c r="J32">
+        <v>11</v>
+      </c>
+      <c r="K32">
+        <v>5</v>
+      </c>
+      <c r="L32">
+        <v>16</v>
+      </c>
+      <c r="M32">
+        <v>20</v>
+      </c>
+      <c r="N32">
+        <v>0</v>
+      </c>
+      <c r="O32">
+        <v>4</v>
+      </c>
+      <c r="P32">
+        <v>0</v>
+      </c>
+      <c r="Q32">
+        <v>72</v>
+      </c>
+      <c r="R32">
+        <v>0</v>
+      </c>
+      <c r="S32">
+        <v>0</v>
+      </c>
+      <c r="T32">
+        <v>16</v>
+      </c>
+      <c r="U32">
+        <v>11</v>
+      </c>
+      <c r="V32">
+        <v>5</v>
+      </c>
+      <c r="W32">
+        <v>0</v>
+      </c>
+      <c r="X32">
+        <v>0</v>
+      </c>
+      <c r="Y32">
+        <v>0</v>
+      </c>
+      <c r="Z32">
+        <v>16</v>
+      </c>
+      <c r="AA32">
+        <v>20</v>
+      </c>
+      <c r="AB32">
+        <v>4</v>
+      </c>
+      <c r="AC32">
+        <v>0</v>
+      </c>
+      <c r="AD32">
+        <v>0</v>
+      </c>
+      <c r="AE32">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_2.jpg</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C33">
+        <v>10497</v>
+      </c>
+      <c r="D33">
+        <v>7549</v>
+      </c>
+      <c r="E33">
+        <v>120</v>
+      </c>
+      <c r="F33">
+        <v>7429</v>
+      </c>
+      <c r="G33">
+        <v>2948</v>
+      </c>
+      <c r="H33">
+        <v>19</v>
+      </c>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <v>35</v>
+      </c>
+      <c r="K33">
+        <v>9</v>
+      </c>
+      <c r="L33">
+        <v>42</v>
+      </c>
+      <c r="M33">
+        <v>20</v>
+      </c>
+      <c r="N33">
+        <v>0</v>
+      </c>
+      <c r="O33">
+        <v>26</v>
+      </c>
+      <c r="P33">
+        <v>0</v>
+      </c>
+      <c r="Q33">
+        <v>151</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>19</v>
+      </c>
+      <c r="U33">
+        <v>35</v>
+      </c>
+      <c r="V33">
+        <v>9</v>
+      </c>
+      <c r="W33">
+        <v>0</v>
+      </c>
+      <c r="X33">
+        <v>0</v>
+      </c>
+      <c r="Y33">
+        <v>0</v>
+      </c>
+      <c r="Z33">
+        <v>42</v>
+      </c>
+      <c r="AA33">
+        <v>20</v>
+      </c>
+      <c r="AB33">
+        <v>26</v>
+      </c>
+      <c r="AC33">
+        <v>0</v>
+      </c>
+      <c r="AD33">
+        <v>0</v>
+      </c>
+      <c r="AE33">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="str">
+        <v>LINE_ALBUM_Sales for September(B1)_261001_1.jpg</v>
+      </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF33"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1060,7 +4153,7 @@
 
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F582"/>
+  <dimension ref="A1:F600"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -12667,10 +15760,369 @@
         <v>14560</v>
       </c>
     </row>
+    <row r="583">
+      <c r="A583" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B583" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C583" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D583" t="str">
+        <v>Watermelon</v>
+      </c>
+      <c r="E583" t="str">
+        <v>แตงโม (evidenced pool 44.6% B1 usage)</v>
+      </c>
+      <c r="F583">
+        <v>22160</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B584" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C584" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D584" t="str">
+        <v>Mango</v>
+      </c>
+      <c r="E584" t="str">
+        <v>มะม่วง (evidenced pool incl IMG_3013.JPG ฿2,750)</v>
+      </c>
+      <c r="F584">
+        <v>21584</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B585" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C585" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D585" t="str">
+        <v>Coconut</v>
+      </c>
+      <c r="E585" t="str">
+        <v>มะพร้าว (evidenced pool 34.0% B1 usage)</v>
+      </c>
+      <c r="F585">
+        <v>11675</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B586" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C586" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D586" t="str">
+        <v>Orange</v>
+      </c>
+      <c r="E586" t="str">
+        <v>ส้ม (evidenced pool 45.2% B1 usage)</v>
+      </c>
+      <c r="F586">
+        <v>10720</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B587" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C587" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D587" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="E587" t="str">
+        <v>สับปะรด (evidenced pool 27.1% B1 usage)</v>
+      </c>
+      <c r="F587">
+        <v>9190</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B588" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C588" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D588" t="str">
+        <v>Apple</v>
+      </c>
+      <c r="E588" t="str">
+        <v>แอปเปิ้ล (evidenced pool 37.4% B1 usage)</v>
+      </c>
+      <c r="F588">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B589" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C589" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D589" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="E589" t="str">
+        <v>ฝรั่ง (evidenced pool 43.9% B1 usage)</v>
+      </c>
+      <c r="F589">
+        <v>6675</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B590" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C590" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D590" t="str">
+        <v>Packaging</v>
+      </c>
+      <c r="E590" t="str">
+        <v>บรรจุภัณฑ์ แก้ว/หลอด/ถุง (pool by rev share)</v>
+      </c>
+      <c r="F590">
+        <v>14143</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B591" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C591" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D591" t="str">
+        <v>Milk/Conden</v>
+      </c>
+      <c r="E591" t="str">
+        <v>นมข้นจืด 2 ลัง (pool by rev share)</v>
+      </c>
+      <c r="F591">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B592" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C592" t="str">
+        <v>COGS</v>
+      </c>
+      <c r="D592" t="str">
+        <v>Other</v>
+      </c>
+      <c r="E592" t="str">
+        <v>วัตถุดิบผลไม้อื่นๆ / Slip 19 ฿5k (pool by rev share)</v>
+      </c>
+      <c r="F592">
+        <v>6860</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="str">
+        <v>03/09/2026</v>
+      </c>
+      <c r="B593" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C593" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D593" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E593" t="str">
+        <v>ค่าเช่าที่ B1 เดือน 9 (Slip 53)</v>
+      </c>
+      <c r="F593">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B594" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C594" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D594" t="str">
+        <v>Rental</v>
+      </c>
+      <c r="E594" t="str">
+        <v>ค่าเช่า storage เดือน 9 (1/4 split B1)</v>
+      </c>
+      <c r="F594">
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B595" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C595" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D595" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E595" t="str">
+        <v>เงินเดือนพนักงาน B1 ก.ย. (Aye 13,500 + Kyaw 12,000)</v>
+      </c>
+      <c r="F595">
+        <v>25500</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>04/09/2026</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C596" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D596" t="str">
+        <v>Salary</v>
+      </c>
+      <c r="E596" t="str">
+        <v>Ming manager wage Sep (1/4 of ฿20,000; Slip 47)</v>
+      </c>
+      <c r="F596">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>30/09/2026</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C597" t="str">
+        <v>OPEX</v>
+      </c>
+      <c r="D597" t="str">
+        <v>Other OPEX</v>
+      </c>
+      <c r="E597" t="str">
+        <v>ค่าขนส่ง / logistics / supplies Sep (B1 portion 37.78%)</v>
+      </c>
+      <c r="F597">
+        <v>4684.34</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>24/09/2026</v>
+      </c>
+      <c r="B598" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C598" t="str">
+        <v>CAPEX</v>
+      </c>
+      <c r="D598" t="str">
+        <v>Equipment</v>
+      </c>
+      <c r="E598" t="str">
+        <v>ค่ามอไซต์ yamaha finn2022 (Slip 73)</v>
+      </c>
+      <c r="F598">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>04/09/2026</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C599" t="str">
+        <v>EXCLUDED</v>
+      </c>
+      <c r="D599" t="str">
+        <v>Personal</v>
+      </c>
+      <c r="E599" t="str">
+        <v>หมูกรอบ 10 โล (Slip 20)</v>
+      </c>
+      <c r="F599">
+        <v>3800</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Sep26</v>
+      </c>
+      <c r="C600" t="str">
+        <v>EXCLUDED</v>
+      </c>
+      <c r="D600" t="str">
+        <v>Internal Transfer</v>
+      </c>
+      <c r="E600" t="str">
+        <v>โอนเงินภายใน (Slip 2: 4,760, Slip 41: 1,275, Slip 70: 3,910)</v>
+      </c>
+      <c r="F600">
+        <v>9945</v>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F582"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F600"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
feat(B2): integrate 20, 21, 22 Sep sales reports into master workbook and dashboard
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -16054,10 +16054,10 @@
         <v>Other OPEX</v>
       </c>
       <c r="E597" t="str">
-        <v>ค่าขนส่ง / logistics / supplies Sep (B1 portion 37.78%)</v>
+        <v>ค่าขนส่ง / logistics / supplies Sep (B1 portion 37.10%)</v>
       </c>
       <c r="F597">
-        <v>4684.34</v>
+        <v>4600.56</v>
       </c>
     </row>
     <row r="598">

</xml_diff>

<commit_message>
Import approved LINE batch set_single636646695303905728
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -136,10 +136,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -171,10 +171,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -3810,7 +3810,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:S4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3872,11 +3872,34 @@
       <c r="R3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
+      <c r="S3" t="str">
+        <v>Source Note</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>01/10/2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C4">
+        <v>5635</v>
+      </c>
+      <c r="D4">
+        <v>3435</v>
+      </c>
+      <c r="G4">
+        <v>2200</v>
+      </c>
+      <c r="S4" t="str">
+        <v>LINE set_single636646695303905728 sha256:4ca01e29ca7b | some cup counts were uncertain and were not written</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Import B1 sales 1-17 Oct 2026 from Parn's photos (approved by Parn)
17 days, revenue 110,471, expenses 2,307. Oct26 sheet moved to the Sep26 column layout; the bot's partial 01/10 row (no cups/ice) is replaced by the full photo row.
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -136,10 +136,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -171,10 +171,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -3810,7 +3810,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S4"/>
+  <dimension ref="A1:AF20"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3843,36 +3843,75 @@
         <v>Orange</v>
       </c>
       <c r="I3" t="str">
+        <v>Orange (100)</v>
+      </c>
+      <c r="J3" t="str">
         <v>Watermelon</v>
       </c>
-      <c r="J3" t="str">
+      <c r="K3" t="str">
         <v>Mango</v>
       </c>
-      <c r="K3" t="str">
+      <c r="L3" t="str">
         <v>Coconut</v>
       </c>
-      <c r="L3" t="str">
+      <c r="M3" t="str">
         <v>Apple</v>
       </c>
-      <c r="M3" t="str">
+      <c r="N3" t="str">
         <v>Young Coco</v>
       </c>
-      <c r="N3" t="str">
+      <c r="O3" t="str">
+        <v>Guava</v>
+      </c>
+      <c r="P3" t="str">
+        <v>Pineapple</v>
+      </c>
+      <c r="Q3" t="str">
         <v>Total Cups</v>
       </c>
-      <c r="O3" t="str">
+      <c r="R3" t="str">
         <v>Bot Big</v>
       </c>
-      <c r="P3" t="str">
+      <c r="S3" t="str">
         <v>Bot Small</v>
       </c>
-      <c r="Q3" t="str">
+      <c r="T3" t="str">
         <v>Used Orange (basket)</v>
       </c>
-      <c r="R3" t="str">
+      <c r="U3" t="str">
         <v>Used Watermelon (pcs)</v>
       </c>
-      <c r="S3" t="str">
+      <c r="V3" t="str">
+        <v>Used Mango</v>
+      </c>
+      <c r="W3" t="str">
+        <v>Used Coco (Meat)</v>
+      </c>
+      <c r="X3" t="str">
+        <v>Used Coco (Water)</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Used Coco (Conden)</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>Used Coco (Raw)</v>
+      </c>
+      <c r="AA3" t="str">
+        <v>Used Apple</v>
+      </c>
+      <c r="AB3" t="str">
+        <v>Used Guava</v>
+      </c>
+      <c r="AC3" t="str">
+        <v>Used Pineapple</v>
+      </c>
+      <c r="AD3" t="str">
+        <v>Used Young Coco</v>
+      </c>
+      <c r="AE3" t="str">
+        <v>Bottle Revenue (฿)</v>
+      </c>
+      <c r="AF3" t="str">
         <v>Source Note</v>
       </c>
     </row>
@@ -3889,17 +3928,801 @@
       <c r="D4">
         <v>3435</v>
       </c>
+      <c r="E4">
+        <v>120</v>
+      </c>
       <c r="G4">
         <v>2200</v>
       </c>
-      <c r="S4" t="str">
-        <v>LINE set_single636646695303905728 sha256:4ca01e29ca7b | some cup counts were uncertain and were not written</v>
+      <c r="H4">
+        <v>10</v>
+      </c>
+      <c r="J4">
+        <v>31</v>
+      </c>
+      <c r="K4">
+        <v>2</v>
+      </c>
+      <c r="L4">
+        <v>21</v>
+      </c>
+      <c r="M4">
+        <v>10</v>
+      </c>
+      <c r="O4">
+        <v>11</v>
+      </c>
+      <c r="P4">
+        <v>5</v>
+      </c>
+      <c r="Q4">
+        <v>90</v>
+      </c>
+      <c r="AF4" t="str">
+        <v>Parn LINE photo 01M56S0550TR12E2KP35RACNK6.jpg (B1 Daily Sales Record 01/10/26), hand-transcribed 2026-10-18</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>02/10/2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C5">
+        <v>7932</v>
+      </c>
+      <c r="D5">
+        <v>4963</v>
+      </c>
+      <c r="E5">
+        <v>243</v>
+      </c>
+      <c r="G5">
+        <v>2969</v>
+      </c>
+      <c r="H5">
+        <v>27</v>
+      </c>
+      <c r="J5">
+        <v>36</v>
+      </c>
+      <c r="K5">
+        <v>5</v>
+      </c>
+      <c r="L5">
+        <v>9</v>
+      </c>
+      <c r="M5">
+        <v>8</v>
+      </c>
+      <c r="O5">
+        <v>21</v>
+      </c>
+      <c r="P5">
+        <v>7</v>
+      </c>
+      <c r="Q5">
+        <v>113</v>
+      </c>
+      <c r="AF5" t="str">
+        <v>Parn LINE photo 01M56S05A5WEC7ZZA3EF92N2J0.jpg (B1 Daily Sales Record 02/10/26), hand-transcribed 2026-10-18</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>03/10/2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C6">
+        <v>7290</v>
+      </c>
+      <c r="D6">
+        <v>4012</v>
+      </c>
+      <c r="E6">
+        <v>165</v>
+      </c>
+      <c r="G6">
+        <v>3278</v>
+      </c>
+      <c r="H6">
+        <v>18</v>
+      </c>
+      <c r="J6">
+        <v>27</v>
+      </c>
+      <c r="K6">
+        <v>3</v>
+      </c>
+      <c r="L6">
+        <v>22</v>
+      </c>
+      <c r="M6">
+        <v>8</v>
+      </c>
+      <c r="O6">
+        <v>17</v>
+      </c>
+      <c r="P6">
+        <v>4</v>
+      </c>
+      <c r="Q6">
+        <v>104</v>
+      </c>
+      <c r="AF6" t="str">
+        <v>Parn LINE photo 01M56RY95HJWHKJDPACECRZDWA.jpg (B1 Daily Sales Record 03/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 2, Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>04/10/2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C7">
+        <v>8297</v>
+      </c>
+      <c r="D7">
+        <v>5124</v>
+      </c>
+      <c r="E7">
+        <v>120</v>
+      </c>
+      <c r="G7">
+        <v>3173</v>
+      </c>
+      <c r="H7">
+        <v>17</v>
+      </c>
+      <c r="J7">
+        <v>40</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>13</v>
+      </c>
+      <c r="M7">
+        <v>10</v>
+      </c>
+      <c r="O7">
+        <v>20</v>
+      </c>
+      <c r="P7">
+        <v>9</v>
+      </c>
+      <c r="Q7">
+        <v>123</v>
+      </c>
+      <c r="AF7" t="str">
+        <v>Parn LINE photo 01M56RY95FA3R8TQDGARQ9K146.jpg (B1 Daily Sales Record 04/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 3, Pomegranate 4 | CHECK: cash items 5,536 vs written 5,124 (+412)</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>05/10/2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C8">
+        <v>7002</v>
+      </c>
+      <c r="D8">
+        <v>4132</v>
+      </c>
+      <c r="E8">
+        <v>120</v>
+      </c>
+      <c r="G8">
+        <v>2870</v>
+      </c>
+      <c r="H8">
+        <v>11</v>
+      </c>
+      <c r="J8">
+        <v>34</v>
+      </c>
+      <c r="K8">
+        <v>8</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8">
+        <v>12</v>
+      </c>
+      <c r="O8">
+        <v>13</v>
+      </c>
+      <c r="P8">
+        <v>5</v>
+      </c>
+      <c r="Q8">
+        <v>90</v>
+      </c>
+      <c r="AF8" t="str">
+        <v>Parn LINE photo 01M56RY95XVEQ7MHKGTWFMS33J.jpg (B1 Daily Sales Record 05/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>06/10/2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C9">
+        <v>7082</v>
+      </c>
+      <c r="D9">
+        <v>4338</v>
+      </c>
+      <c r="E9">
+        <v>120</v>
+      </c>
+      <c r="G9">
+        <v>2744</v>
+      </c>
+      <c r="H9">
+        <v>16</v>
+      </c>
+      <c r="J9">
+        <v>40</v>
+      </c>
+      <c r="K9">
+        <v>6</v>
+      </c>
+      <c r="L9">
+        <v>9</v>
+      </c>
+      <c r="M9">
+        <v>5</v>
+      </c>
+      <c r="O9">
+        <v>20</v>
+      </c>
+      <c r="P9">
+        <v>0</v>
+      </c>
+      <c r="Q9">
+        <v>102</v>
+      </c>
+      <c r="AF9" t="str">
+        <v>Parn LINE photo 01M56RY947GB54Y6M8KYPK4Y0Q.jpg (B1 Daily Sales Record 06/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 2, Pomegranate 4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>07/10/2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C10">
+        <v>4134</v>
+      </c>
+      <c r="D10">
+        <v>2754</v>
+      </c>
+      <c r="E10">
+        <v>60</v>
+      </c>
+      <c r="G10">
+        <v>1380</v>
+      </c>
+      <c r="H10">
+        <v>11</v>
+      </c>
+      <c r="J10">
+        <v>14</v>
+      </c>
+      <c r="K10">
+        <v>2</v>
+      </c>
+      <c r="L10">
+        <v>12</v>
+      </c>
+      <c r="M10">
+        <v>5</v>
+      </c>
+      <c r="O10">
+        <v>6</v>
+      </c>
+      <c r="P10">
+        <v>0</v>
+      </c>
+      <c r="Q10">
+        <v>57</v>
+      </c>
+      <c r="AF10" t="str">
+        <v>Parn LINE photo 01M56S04V94F0F0YH6T7N5KGJJ.jpg (B1 Daily Sales Record 07/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 3, Pomegranate 4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>08/10/2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C11">
+        <v>3896</v>
+      </c>
+      <c r="D11">
+        <v>2716</v>
+      </c>
+      <c r="E11">
+        <v>180</v>
+      </c>
+      <c r="G11">
+        <v>1180</v>
+      </c>
+      <c r="H11">
+        <v>10</v>
+      </c>
+      <c r="J11">
+        <v>18</v>
+      </c>
+      <c r="K11">
+        <v>4</v>
+      </c>
+      <c r="L11">
+        <v>3</v>
+      </c>
+      <c r="M11">
+        <v>6</v>
+      </c>
+      <c r="O11">
+        <v>8</v>
+      </c>
+      <c r="P11">
+        <v>0</v>
+      </c>
+      <c r="Q11">
+        <v>52</v>
+      </c>
+      <c r="AF11" t="str">
+        <v>Parn LINE photo 01M56S04WAYMK805PMJ7273F3W.jpg (B1 Daily Sales Record 08/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 3</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>09/10/2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C12">
+        <v>5393</v>
+      </c>
+      <c r="D12">
+        <v>2912</v>
+      </c>
+      <c r="E12">
+        <v>120</v>
+      </c>
+      <c r="G12">
+        <v>2481</v>
+      </c>
+      <c r="H12">
+        <v>11</v>
+      </c>
+      <c r="J12">
+        <v>30</v>
+      </c>
+      <c r="K12">
+        <v>4</v>
+      </c>
+      <c r="L12">
+        <v>7</v>
+      </c>
+      <c r="M12">
+        <v>6</v>
+      </c>
+      <c r="O12">
+        <v>9</v>
+      </c>
+      <c r="P12">
+        <v>0</v>
+      </c>
+      <c r="Q12">
+        <v>72</v>
+      </c>
+      <c r="AF12" t="str">
+        <v>Parn LINE photo 01M56S03NH3PQ120WQZZBC0TEC.jpg (B1 Daily Sales Record 09/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>10/10/2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C13">
+        <v>13333</v>
+      </c>
+      <c r="D13">
+        <v>7450</v>
+      </c>
+      <c r="E13">
+        <v>150</v>
+      </c>
+      <c r="G13">
+        <v>5883</v>
+      </c>
+      <c r="H13">
+        <v>39</v>
+      </c>
+      <c r="J13">
+        <v>70</v>
+      </c>
+      <c r="K13">
+        <v>9</v>
+      </c>
+      <c r="L13">
+        <v>17</v>
+      </c>
+      <c r="M13">
+        <v>17</v>
+      </c>
+      <c r="O13">
+        <v>25</v>
+      </c>
+      <c r="P13">
+        <v>0</v>
+      </c>
+      <c r="Q13">
+        <v>188</v>
+      </c>
+      <c r="AF13" t="str">
+        <v>Parn LINE photo 01M56S03KMN1DWS0GMVJZNPSHP.jpg (B1 Daily Sales Record 10/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 2, Pomegranate 9</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>11/10/2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Sun</v>
+      </c>
+      <c r="C14">
+        <v>9400</v>
+      </c>
+      <c r="D14">
+        <v>6600</v>
+      </c>
+      <c r="E14">
+        <v>369</v>
+      </c>
+      <c r="G14">
+        <v>2800</v>
+      </c>
+      <c r="H14">
+        <v>26</v>
+      </c>
+      <c r="I14">
+        <v>1</v>
+      </c>
+      <c r="J14">
+        <v>37</v>
+      </c>
+      <c r="K14">
+        <v>5</v>
+      </c>
+      <c r="L14">
+        <v>17</v>
+      </c>
+      <c r="M14">
+        <v>10</v>
+      </c>
+      <c r="O14">
+        <v>25</v>
+      </c>
+      <c r="P14">
+        <v>0</v>
+      </c>
+      <c r="Q14">
+        <v>132</v>
+      </c>
+      <c r="AF14" t="str">
+        <v>Parn LINE photo 01M56S00P3CVQASJ77HCCEPXGD.jpg (B1 Daily Sales Record 11/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 10, Grape 2 | CHECK: cash items 6,710 vs written 6,600 (+110)</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>12/10/2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Mon</v>
+      </c>
+      <c r="C15">
+        <v>5172</v>
+      </c>
+      <c r="D15">
+        <v>4023</v>
+      </c>
+      <c r="E15">
+        <v>60</v>
+      </c>
+      <c r="G15">
+        <v>1149</v>
+      </c>
+      <c r="H15">
+        <v>8</v>
+      </c>
+      <c r="J15">
+        <v>32</v>
+      </c>
+      <c r="K15">
+        <v>2</v>
+      </c>
+      <c r="L15">
+        <v>14</v>
+      </c>
+      <c r="M15">
+        <v>7</v>
+      </c>
+      <c r="O15">
+        <v>4</v>
+      </c>
+      <c r="P15">
+        <v>0</v>
+      </c>
+      <c r="Q15">
+        <v>74</v>
+      </c>
+      <c r="AF15" t="str">
+        <v>Parn LINE photo 01M56S03277KX92E9V8AAXVSXR.jpg (B1 Daily Sales Record 12/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 5, Grape 2</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>13/10/2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Tue</v>
+      </c>
+      <c r="C16">
+        <v>6963</v>
+      </c>
+      <c r="D16">
+        <v>4299</v>
+      </c>
+      <c r="E16">
+        <v>120</v>
+      </c>
+      <c r="G16">
+        <v>2664</v>
+      </c>
+      <c r="H16">
+        <v>15</v>
+      </c>
+      <c r="J16">
+        <v>31</v>
+      </c>
+      <c r="K16">
+        <v>2</v>
+      </c>
+      <c r="L16">
+        <v>10</v>
+      </c>
+      <c r="M16">
+        <v>8</v>
+      </c>
+      <c r="O16">
+        <v>13</v>
+      </c>
+      <c r="P16">
+        <v>0</v>
+      </c>
+      <c r="Q16">
+        <v>91</v>
+      </c>
+      <c r="AF16" t="str">
+        <v>Parn LINE photo 01M56S00P08B4VVHAER9EBNT2B.jpg (B1 Daily Sales Record 13/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 9, Grape 1, Pome no ice 2</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>14/10/2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Wed</v>
+      </c>
+      <c r="C17">
+        <v>3105</v>
+      </c>
+      <c r="D17">
+        <v>1600</v>
+      </c>
+      <c r="E17">
+        <v>60</v>
+      </c>
+      <c r="G17">
+        <v>1505</v>
+      </c>
+      <c r="H17">
+        <v>7</v>
+      </c>
+      <c r="J17">
+        <v>22</v>
+      </c>
+      <c r="K17">
+        <v>3</v>
+      </c>
+      <c r="L17">
+        <v>3</v>
+      </c>
+      <c r="M17">
+        <v>8</v>
+      </c>
+      <c r="O17">
+        <v>11</v>
+      </c>
+      <c r="P17">
+        <v>0</v>
+      </c>
+      <c r="Q17">
+        <v>54</v>
+      </c>
+      <c r="AF17" t="str">
+        <v>Parn LINE photo 01M56S00PM4MPZHGK66S1024F3.jpg (B1 Daily Sales Record 14/10/26), hand-transcribed 2026-10-18 | CHECK: cash items 1,908 vs written 1,600 (+308); QR items 1,630 vs written 1,505 (+125)</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>15/10/2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Thu</v>
+      </c>
+      <c r="C18">
+        <v>6101</v>
+      </c>
+      <c r="D18">
+        <v>4053</v>
+      </c>
+      <c r="E18">
+        <v>120</v>
+      </c>
+      <c r="G18">
+        <v>2048</v>
+      </c>
+      <c r="H18">
+        <v>16</v>
+      </c>
+      <c r="J18">
+        <v>31</v>
+      </c>
+      <c r="K18">
+        <v>7</v>
+      </c>
+      <c r="L18">
+        <v>8</v>
+      </c>
+      <c r="M18">
+        <v>4</v>
+      </c>
+      <c r="O18">
+        <v>10</v>
+      </c>
+      <c r="P18">
+        <v>0</v>
+      </c>
+      <c r="Q18">
+        <v>82</v>
+      </c>
+      <c r="AF18" t="str">
+        <v>Parn LINE photo 01M56S00NX7K0QAGGESZ99F5HN.jpg (B1 Daily Sales Record 15/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Pomegranate 6</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>16/10/2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Fri</v>
+      </c>
+      <c r="C19">
+        <v>3090</v>
+      </c>
+      <c r="D19">
+        <v>1965</v>
+      </c>
+      <c r="E19">
+        <v>120</v>
+      </c>
+      <c r="G19">
+        <v>1125</v>
+      </c>
+      <c r="H19">
+        <v>8</v>
+      </c>
+      <c r="J19">
+        <v>11</v>
+      </c>
+      <c r="K19">
+        <v>2</v>
+      </c>
+      <c r="L19">
+        <v>3</v>
+      </c>
+      <c r="M19">
+        <v>7</v>
+      </c>
+      <c r="O19">
+        <v>15</v>
+      </c>
+      <c r="P19">
+        <v>0</v>
+      </c>
+      <c r="Q19">
+        <v>47</v>
+      </c>
+      <c r="AF19" t="str">
+        <v>Parn LINE photo 01M56S00KKXF5PZNYAWYP4CRCE.jpg (B1 Daily Sales Record 16/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 1 | CHECK: cash items 2,009 vs written 1,965 (+44)</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>17/10/2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Sat</v>
+      </c>
+      <c r="C20">
+        <v>6646</v>
+      </c>
+      <c r="D20">
+        <v>4077</v>
+      </c>
+      <c r="E20">
+        <v>60</v>
+      </c>
+      <c r="G20">
+        <v>2569</v>
+      </c>
+      <c r="H20">
+        <v>15</v>
+      </c>
+      <c r="I20">
+        <v>1</v>
+      </c>
+      <c r="J20">
+        <v>21</v>
+      </c>
+      <c r="K20">
+        <v>2</v>
+      </c>
+      <c r="L20">
+        <v>16</v>
+      </c>
+      <c r="M20">
+        <v>8</v>
+      </c>
+      <c r="O20">
+        <v>19</v>
+      </c>
+      <c r="P20">
+        <v>0</v>
+      </c>
+      <c r="Q20">
+        <v>89</v>
+      </c>
+      <c r="AF20" t="str">
+        <v>Parn LINE photo 01M56S00P1Q25BFZ7DMKJ45R96.jpg (B1 Daily Sales Record 17/10/26), hand-transcribed 2026-10-18 | not in fruit columns: Grape 1, Pomegranate 6, Pome no ice 1</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AF20"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Used fruit columns: B4 Sep Used fixed (mangosteen out of Used Mango, pineapple), B1 Sep pineapple/watermelon re-booked from the sheets; book the written fruit (approved by Parn)
</commit_message>
<xml_diff>
--- a/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
+++ b/3_Automation_Dashboard/SomSaiJai_Dashboard_B1_2026.xlsx
@@ -136,10 +136,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -171,10 +171,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -1291,7 +1291,7 @@
         <v>8</v>
       </c>
       <c r="M8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -1300,7 +1300,7 @@
         <v>6</v>
       </c>
       <c r="P8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q8">
         <v>85</v>
@@ -1333,13 +1333,13 @@
         <v>8</v>
       </c>
       <c r="AA8">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AB8">
         <v>6</v>
       </c>
       <c r="AC8">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD8">
         <v>0</v>
@@ -1683,7 +1683,7 @@
         <v>7</v>
       </c>
       <c r="M12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N12">
         <v>0</v>
@@ -1692,7 +1692,7 @@
         <v>3</v>
       </c>
       <c r="P12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12">
         <v>67</v>
@@ -1725,13 +1725,13 @@
         <v>7</v>
       </c>
       <c r="AA12">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB12">
         <v>3</v>
       </c>
       <c r="AC12">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD12">
         <v>0</v>
@@ -2173,7 +2173,7 @@
         <v>11</v>
       </c>
       <c r="M17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N17">
         <v>0</v>
@@ -2182,7 +2182,7 @@
         <v>4</v>
       </c>
       <c r="P17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q17">
         <v>68</v>
@@ -2215,13 +2215,13 @@
         <v>11</v>
       </c>
       <c r="AA17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB17">
         <v>4</v>
       </c>
       <c r="AC17">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AD17">
         <v>0</v>
@@ -2458,16 +2458,16 @@
         <v>0</v>
       </c>
       <c r="J20">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="M20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N20">
         <v>0</v>
@@ -2476,7 +2476,7 @@
         <v>2</v>
       </c>
       <c r="P20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q20">
         <v>29</v>
@@ -2491,7 +2491,7 @@
         <v>10</v>
       </c>
       <c r="U20">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="V20">
         <v>0</v>
@@ -2506,16 +2506,16 @@
         <v>0</v>
       </c>
       <c r="Z20">
-        <v>11</v>
+        <v>0</v>
       </c>
       <c r="AA20">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AB20">
         <v>2</v>
       </c>
       <c r="AC20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD20">
         <v>0</v>
@@ -2556,16 +2556,16 @@
         <v>0</v>
       </c>
       <c r="J21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K21">
         <v>3</v>
       </c>
       <c r="L21">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="M21">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="N21">
         <v>0</v>
@@ -2574,7 +2574,7 @@
         <v>10</v>
       </c>
       <c r="P21">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="Q21">
         <v>73</v>
@@ -2589,7 +2589,7 @@
         <v>14</v>
       </c>
       <c r="U21">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="V21">
         <v>3</v>
@@ -2604,16 +2604,16 @@
         <v>0</v>
       </c>
       <c r="Z21">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="AA21">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="AB21">
         <v>10</v>
       </c>
       <c r="AC21">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="AD21">
         <v>0</v>
@@ -2663,7 +2663,7 @@
         <v>12</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N22">
         <v>0</v>
@@ -2672,7 +2672,7 @@
         <v>6</v>
       </c>
       <c r="P22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q22">
         <v>48</v>
@@ -2705,13 +2705,13 @@
         <v>12</v>
       </c>
       <c r="AA22">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="AB22">
         <v>6</v>
       </c>
       <c r="AC22">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD22">
         <v>0</v>
@@ -2752,16 +2752,16 @@
         <v>0</v>
       </c>
       <c r="J23">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="K23">
         <v>1</v>
       </c>
       <c r="L23">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="M23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="N23">
         <v>0</v>
@@ -2770,7 +2770,7 @@
         <v>1</v>
       </c>
       <c r="P23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q23">
         <v>15</v>
@@ -2785,7 +2785,7 @@
         <v>2</v>
       </c>
       <c r="U23">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="V23">
         <v>1</v>
@@ -2800,16 +2800,16 @@
         <v>0</v>
       </c>
       <c r="Z23">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AA23">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AB23">
         <v>1</v>
       </c>
       <c r="AC23">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AD23">
         <v>0</v>
@@ -2859,7 +2859,7 @@
         <v>10</v>
       </c>
       <c r="M24">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="N24">
         <v>0</v>
@@ -2868,7 +2868,7 @@
         <v>4</v>
       </c>
       <c r="P24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q24">
         <v>41</v>
@@ -2901,13 +2901,13 @@
         <v>10</v>
       </c>
       <c r="AA24">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AB24">
         <v>4</v>
       </c>
       <c r="AC24">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD24">
         <v>0</v>
@@ -2948,16 +2948,16 @@
         <v>0</v>
       </c>
       <c r="J25">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="K25">
         <v>2</v>
       </c>
       <c r="L25">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="M25">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="N25">
         <v>0</v>
@@ -2966,7 +2966,7 @@
         <v>6</v>
       </c>
       <c r="P25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q25">
         <v>61</v>
@@ -2981,7 +2981,7 @@
         <v>12</v>
       </c>
       <c r="U25">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="V25">
         <v>2</v>
@@ -2996,16 +2996,16 @@
         <v>0</v>
       </c>
       <c r="Z25">
-        <v>29</v>
+        <v>5</v>
       </c>
       <c r="AA25">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="AB25">
         <v>6</v>
       </c>
       <c r="AC25">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD25">
         <v>0</v>
@@ -3046,13 +3046,13 @@
         <v>0</v>
       </c>
       <c r="J26">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="K26">
         <v>10</v>
       </c>
       <c r="L26">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="M26">
         <v>4</v>
@@ -3079,7 +3079,7 @@
         <v>6</v>
       </c>
       <c r="U26">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="V26">
         <v>10</v>
@@ -3094,7 +3094,7 @@
         <v>0</v>
       </c>
       <c r="Z26">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="AA26">
         <v>4</v>
@@ -3153,7 +3153,7 @@
         <v>6</v>
       </c>
       <c r="M27">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="N27">
         <v>0</v>
@@ -3162,7 +3162,7 @@
         <v>5</v>
       </c>
       <c r="P27">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="Q27">
         <v>47</v>
@@ -3195,13 +3195,13 @@
         <v>6</v>
       </c>
       <c r="AA27">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="AB27">
         <v>5</v>
       </c>
       <c r="AC27">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AD27">
         <v>0</v>
@@ -3349,7 +3349,7 @@
         <v>14</v>
       </c>
       <c r="M29">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N29">
         <v>0</v>
@@ -3358,7 +3358,7 @@
         <v>11</v>
       </c>
       <c r="P29">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="Q29">
         <v>99</v>
@@ -3391,13 +3391,13 @@
         <v>14</v>
       </c>
       <c r="AA29">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="AB29">
         <v>11</v>
       </c>
       <c r="AC29">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="AD29">
         <v>0</v>
@@ -3447,7 +3447,7 @@
         <v>9</v>
       </c>
       <c r="M30">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="N30">
         <v>0</v>
@@ -3456,7 +3456,7 @@
         <v>9</v>
       </c>
       <c r="P30">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="Q30">
         <v>77</v>
@@ -3489,13 +3489,13 @@
         <v>9</v>
       </c>
       <c r="AA30">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="AB30">
         <v>9</v>
       </c>
       <c r="AC30">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="AD30">
         <v>0</v>
@@ -3545,7 +3545,7 @@
         <v>5</v>
       </c>
       <c r="M31">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="N31">
         <v>0</v>
@@ -3554,7 +3554,7 @@
         <v>12</v>
       </c>
       <c r="P31">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="Q31">
         <v>71</v>
@@ -3587,13 +3587,13 @@
         <v>5</v>
       </c>
       <c r="AA31">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AB31">
         <v>12</v>
       </c>
       <c r="AC31">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AD31">
         <v>0</v>
@@ -3643,7 +3643,7 @@
         <v>16</v>
       </c>
       <c r="M32">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N32">
         <v>0</v>
@@ -3652,7 +3652,7 @@
         <v>4</v>
       </c>
       <c r="P32">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="Q32">
         <v>72</v>
@@ -3685,13 +3685,13 @@
         <v>16</v>
       </c>
       <c r="AA32">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="AB32">
         <v>4</v>
       </c>
       <c r="AC32">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AD32">
         <v>0</v>
@@ -3732,16 +3732,16 @@
         <v>0</v>
       </c>
       <c r="J33">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="K33">
         <v>9</v>
       </c>
       <c r="L33">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="M33">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="N33">
         <v>0</v>
@@ -3750,7 +3750,7 @@
         <v>26</v>
       </c>
       <c r="P33">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="Q33">
         <v>151</v>
@@ -3765,7 +3765,7 @@
         <v>19</v>
       </c>
       <c r="U33">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="V33">
         <v>9</v>
@@ -3780,16 +3780,16 @@
         <v>0</v>
       </c>
       <c r="Z33">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="AA33">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="AB33">
         <v>26</v>
       </c>
       <c r="AC33">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="AD33">
         <v>0</v>

</xml_diff>